<commit_message>
Update pricing logic, UI formatting and PDF generation features
</commit_message>
<xml_diff>
--- a/data/quan ly don hang HLK.xlsx
+++ b/data/quan ly don hang HLK.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12570" activeTab="4"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12570" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="MENU" sheetId="14" r:id="rId1"/>
@@ -893,7 +893,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -939,6 +939,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1067,7 +1073,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1227,12 +1233,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1251,9 +1251,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1297,7 +1316,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1361,7 +1380,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1425,7 +1444,7 @@
           <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1494,7 +1513,7 @@
         <xdr:cNvPr id="2" name="Rounded Rectangle 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0100-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1562,7 +1581,7 @@
         <xdr:cNvPr id="2" name="Rounded Rectangle 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0200-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1630,7 +1649,7 @@
         <xdr:cNvPr id="2" name="Rounded Rectangle 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0300-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2014,81 +2033,81 @@
       <c r="L3" s="1"/>
     </row>
     <row r="4" spans="3:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="C4" s="2">
+      <c r="C4" s="64">
         <v>1</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="14" t="str">
+      <c r="E4" s="66" t="str">
         <f>VLOOKUP(D4,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bulong Đầu Bông Thép Mạ Kẽm 10.9 DIN6921 M10x20 (Có Khía)</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="64">
         <v>5</v>
       </c>
-      <c r="G4" s="4" t="str">
+      <c r="G4" s="67" t="str">
         <f>VLOOKUP(D4,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Cái</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="39" t="s">
+      <c r="I4" s="68" t="s">
         <v>101</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
     </row>
     <row r="5" spans="3:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="C5" s="2">
+      <c r="C5" s="64">
         <v>2</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="14" t="str">
+      <c r="E5" s="66" t="str">
         <f>VLOOKUP(D5,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Khía Thép Mạ Kẽm 8.8 DIN6923 M10</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="64">
         <v>5</v>
       </c>
-      <c r="G5" s="4" t="str">
+      <c r="G5" s="67" t="str">
         <f>VLOOKUP(D5,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Cái</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="I5" s="39" t="s">
+      <c r="I5" s="68" t="s">
         <v>101</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
     </row>
     <row r="6" spans="3:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="C6" s="2">
+      <c r="C6" s="64">
         <v>3</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="65" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="14" t="str">
+      <c r="E6" s="66" t="str">
         <f>VLOOKUP(D6,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Thước Cặp Cơ Khí 0-150mm/0-6inch INSIZE 1205-1502S</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="64">
         <v>1</v>
       </c>
-      <c r="G6" s="4" t="str">
+      <c r="G6" s="67" t="str">
         <f>VLOOKUP(D6,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Cái</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="I6" s="39" t="s">
+      <c r="I6" s="68" t="s">
         <v>101</v>
       </c>
       <c r="K6" s="1"/>
@@ -6622,27 +6641,27 @@
       </c>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="3:11" ht="18" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:11" ht="18.75" x14ac:dyDescent="0.25">
       <c r="C6" s="2">
         <v>1</v>
       </c>
-      <c r="D6" s="22" t="str">
+      <c r="D6" s="65" t="str">
         <f>'danh mục Vật tư'!B3</f>
         <v>B08M1001020TE20</v>
       </c>
-      <c r="E6" s="2" t="str">
+      <c r="E6" s="64" t="str">
         <f>VLOOKUP(D6,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bulong Đầu Bông Thép Mạ Kẽm 10.9 DIN6921 M10x20 (Có Khía)</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D6,Nhập!$F$4:$F$1213)</f>
         <v>5</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D6,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="64">
         <f>F6-G6</f>
         <v>5</v>
       </c>
@@ -6657,23 +6676,23 @@
       <c r="C7" s="2">
         <v>2</v>
       </c>
-      <c r="D7" s="22" t="str">
+      <c r="D7" s="65" t="str">
         <f>'danh mục Vật tư'!B4</f>
         <v>N02M1001D21</v>
       </c>
-      <c r="E7" s="2" t="str">
+      <c r="E7" s="64" t="str">
         <f>VLOOKUP(D7,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Khía Thép Mạ Kẽm 8.8 DIN6923 M10</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D7,Nhập!$F$4:$F$1213)</f>
         <v>5</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D7,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="64">
         <f t="shared" ref="H7:H20" si="0">F7-G7</f>
         <v>5</v>
       </c>
@@ -6688,23 +6707,23 @@
       <c r="C8" s="2">
         <v>3</v>
       </c>
-      <c r="D8" s="22" t="str">
+      <c r="D8" s="65" t="str">
         <f>'danh mục Vật tư'!B5</f>
         <v>INS-1205-1502S</v>
       </c>
-      <c r="E8" s="2" t="str">
+      <c r="E8" s="64" t="str">
         <f>VLOOKUP(D8,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Thước Cặp Cơ Khí 0-150mm/0-6inch INSIZE 1205-1502S</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D8,Nhập!$F$4:$F$1213)</f>
         <v>1</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D8,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="64">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -6719,23 +6738,23 @@
       <c r="C9" s="2">
         <v>4</v>
       </c>
-      <c r="D9" s="22" t="str">
+      <c r="D9" s="65" t="str">
         <f>'danh mục Vật tư'!B6</f>
         <v>N01M0801H00</v>
       </c>
-      <c r="E9" s="2" t="str">
+      <c r="E9" s="64" t="str">
         <f>VLOOKUP(D9,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Inox 304 DIN934 M8</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D9,Nhập!$F$4:$F$1213)</f>
         <v>4900</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D9,Xuất!$F$6:$F$1043)</f>
         <v>1000</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="64">
         <f t="shared" si="0"/>
         <v>3900</v>
       </c>
@@ -6750,23 +6769,23 @@
       <c r="C10" s="2">
         <v>5</v>
       </c>
-      <c r="D10" s="22" t="str">
+      <c r="D10" s="65" t="str">
         <f>'danh mục Vật tư'!B7</f>
         <v>W01M080CH0</v>
       </c>
-      <c r="E10" s="2" t="str">
+      <c r="E10" s="64" t="str">
         <f>VLOOKUP(D10,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Lông Đền Phẳng Inox 304 M8 (19x2.0)</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D10,Nhập!$F$4:$F$1213)</f>
         <v>872</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D10,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="64">
         <f t="shared" si="0"/>
         <v>872</v>
       </c>
@@ -6781,23 +6800,23 @@
       <c r="C11" s="2">
         <v>6</v>
       </c>
-      <c r="D11" s="22" t="str">
+      <c r="D11" s="65" t="str">
         <f>'danh mục Vật tư'!B8</f>
         <v>V0942012B1000</v>
       </c>
-      <c r="E11" s="2" t="str">
+      <c r="E11" s="64" t="str">
         <f>VLOOKUP(D11,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Rivet Nhôm OD4.0x12.7mm (995-1000 Cái)</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D11,Nhập!$F$4:$F$1213)</f>
         <v>1</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D11,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="64">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -6812,23 +6831,23 @@
       <c r="C12" s="2">
         <v>7</v>
       </c>
-      <c r="D12" s="22" t="str">
+      <c r="D12" s="65" t="str">
         <f>'danh mục Vật tư'!B9</f>
         <v>V1140016H100</v>
       </c>
-      <c r="E12" s="2" t="str">
+      <c r="E12" s="64" t="str">
         <f>VLOOKUP(D12,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Rivet Inox 304 OD4.0x16mm (100 Cái)</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D12,Nhập!$F$4:$F$1213)</f>
         <v>1</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D12,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="64">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -6842,23 +6861,23 @@
       <c r="C13" s="2">
         <v>8</v>
       </c>
-      <c r="D13" s="22" t="str">
+      <c r="D13" s="65" t="str">
         <f>'danh mục Vật tư'!B10</f>
         <v>N03M0801H00</v>
       </c>
-      <c r="E13" s="2" t="str">
+      <c r="E13" s="64" t="str">
         <f>VLOOKUP(D13,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Keo Inox 304 DIN985 M8</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F13" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D13,Nhập!$F$4:$F$1213)</f>
         <v>3400</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D13,Xuất!$F$6:$F$1043)</f>
         <v>1400</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="64">
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
@@ -6872,23 +6891,23 @@
       <c r="C14" s="2">
         <v>9</v>
       </c>
-      <c r="D14" s="22" t="str">
+      <c r="D14" s="65" t="str">
         <f>'danh mục Vật tư'!B11</f>
         <v>B01M0801020TH00</v>
       </c>
-      <c r="E14" s="2" t="str">
+      <c r="E14" s="64" t="str">
         <f>VLOOKUP(D14,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bulong Inox 304 DIN933 M8x20</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D14,Nhập!$F$4:$F$1213)</f>
         <v>2550</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D14,Xuất!$F$6:$F$1043)</f>
         <v>1400</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="64">
         <f t="shared" si="0"/>
         <v>1150</v>
       </c>
@@ -6902,23 +6921,23 @@
       <c r="C15" s="2">
         <v>10</v>
       </c>
-      <c r="D15" s="22" t="str">
+      <c r="D15" s="65" t="str">
         <f>'danh mục Vật tư'!B12</f>
         <v>1103N0042</v>
       </c>
-      <c r="E15" s="2" t="str">
+      <c r="E15" s="64" t="str">
         <f>VLOOKUP(D15,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Mũi Khoan Thép List 500 Nachi D4.2</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D15,Nhập!$F$4:$F$1213)</f>
         <v>3</v>
       </c>
-      <c r="G15" s="2">
+      <c r="G15" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D15,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="64">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
@@ -6932,23 +6951,23 @@
       <c r="C16" s="2">
         <v>11</v>
       </c>
-      <c r="D16" s="22" t="str">
+      <c r="D16" s="65" t="str">
         <f>'danh mục Vật tư'!B13</f>
         <v>B01M0801030TD21</v>
       </c>
-      <c r="E16" s="2" t="str">
+      <c r="E16" s="64" t="str">
         <f>VLOOKUP(D16,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bulong Mạ Kẽm 8.8 DIN933 M8x30</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D16,Nhập!$F$4:$F$1213)</f>
         <v>1305</v>
       </c>
-      <c r="G16" s="2">
+      <c r="G16" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D16,Xuất!$F$6:$F$1043)</f>
         <v>1300</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="64">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -6962,23 +6981,23 @@
       <c r="C17" s="2">
         <v>12</v>
       </c>
-      <c r="D17" s="22" t="str">
+      <c r="D17" s="65" t="str">
         <f>'danh mục Vật tư'!B14</f>
         <v>66-119</v>
       </c>
-      <c r="E17" s="2" t="str">
+      <c r="E17" s="64" t="str">
         <f>VLOOKUP(D17,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bút Thử Điện 150mm (100-500V) Stanley 66-119</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D17,Nhập!$F$4:$F$1213)</f>
         <v>5</v>
       </c>
-      <c r="G17" s="2">
+      <c r="G17" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D17,Xuất!$F$6:$F$1043)</f>
         <v>5</v>
       </c>
-      <c r="H17" s="7">
+      <c r="H17" s="64">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -6992,23 +7011,23 @@
       <c r="C18" s="2">
         <v>13</v>
       </c>
-      <c r="D18" s="22" t="str">
+      <c r="D18" s="65" t="str">
         <f>'danh mục Vật tư'!B15</f>
         <v>DACT200-048B</v>
       </c>
-      <c r="E18" s="2" t="str">
+      <c r="E18" s="64" t="str">
         <f>VLOOKUP(D18,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Dây Rút Nhựa Chống Tia UV Màu Đen DONG-A 200x4.8mm (1000 Sợi/Bịch)</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D18,Nhập!$F$4:$F$1213)</f>
         <v>1</v>
       </c>
-      <c r="G18" s="2">
+      <c r="G18" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D18,Xuất!$F$6:$F$1043)</f>
         <v>1</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="64">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -7018,27 +7037,27 @@
       </c>
       <c r="J18" s="22"/>
     </row>
-    <row r="19" spans="3:11" ht="18" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:11" ht="18.75" x14ac:dyDescent="0.25">
       <c r="C19" s="2">
         <v>14</v>
       </c>
-      <c r="D19" s="22" t="str">
+      <c r="D19" s="65" t="str">
         <f>'danh mục Vật tư'!B16</f>
         <v>B03M1001080TK00</v>
       </c>
-      <c r="E19" s="2" t="str">
+      <c r="E19" s="64" t="str">
         <f>VLOOKUP(D19,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Lục Giác Chìm Col Inox 316 DIN7991 M10x80</v>
       </c>
-      <c r="F19" s="2">
+      <c r="F19" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D19,Nhập!$F$4:$F$1213)</f>
         <v>665</v>
       </c>
-      <c r="G19" s="2">
+      <c r="G19" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D19,Xuất!$F$6:$F$1043)</f>
         <v>300</v>
       </c>
-      <c r="H19" s="7">
+      <c r="H19" s="64">
         <f t="shared" si="0"/>
         <v>365</v>
       </c>
@@ -7052,23 +7071,23 @@
       <c r="C20" s="2">
         <v>15</v>
       </c>
-      <c r="D20" s="22" t="str">
+      <c r="D20" s="65" t="str">
         <f>'danh mục Vật tư'!B17</f>
         <v>84-369</v>
       </c>
-      <c r="E20" s="2" t="str">
+      <c r="E20" s="64" t="str">
         <f>VLOOKUP(D20,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Kìm Bấm Chết 10Inch/254mm Stanley 84-369</v>
       </c>
-      <c r="F20" s="2">
+      <c r="F20" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D20,Nhập!$F$4:$F$1213)</f>
         <v>4</v>
       </c>
-      <c r="G20" s="2">
+      <c r="G20" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D20,Xuất!$F$6:$F$1043)</f>
         <v>4</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="64">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -7082,23 +7101,23 @@
       <c r="C21" s="2">
         <v>16</v>
       </c>
-      <c r="D21" s="22" t="str">
+      <c r="D21" s="65" t="str">
         <f>'danh mục Vật tư'!B18</f>
         <v>B01M1201030TH00</v>
       </c>
-      <c r="E21" s="2" t="str">
+      <c r="E21" s="64" t="str">
         <f>VLOOKUP(D21,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bulong Inox 304 DIN933 M12x30</v>
       </c>
-      <c r="F21" s="2">
+      <c r="F21" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D21,Nhập!$F$4:$F$1213)</f>
         <v>1110</v>
       </c>
-      <c r="G21" s="2">
+      <c r="G21" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D21,Xuất!$F$6:$F$1043)</f>
         <v>500</v>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="64">
         <f t="shared" ref="H21:H22" si="1">F21-G21</f>
         <v>610</v>
       </c>
@@ -7112,23 +7131,23 @@
       <c r="C22" s="2">
         <v>17</v>
       </c>
-      <c r="D22" s="22" t="str">
+      <c r="D22" s="65" t="str">
         <f>'danh mục Vật tư'!B19</f>
         <v>N03M1201H00</v>
       </c>
-      <c r="E22" s="2" t="str">
+      <c r="E22" s="64" t="str">
         <f>VLOOKUP(D22,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Keo Inox 304 DIN985 M12</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D22,Nhập!$F$4:$F$1213)</f>
         <v>1905</v>
       </c>
-      <c r="G22" s="2">
+      <c r="G22" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D22,Xuất!$F$6:$F$1043)</f>
         <v>500</v>
       </c>
-      <c r="H22" s="7">
+      <c r="H22" s="64">
         <f t="shared" si="1"/>
         <v>1405</v>
       </c>
@@ -7142,23 +7161,23 @@
       <c r="C23" s="2">
         <v>18</v>
       </c>
-      <c r="D23" s="22" t="str">
+      <c r="D23" s="65" t="str">
         <f>'danh mục Vật tư'!B20</f>
         <v>W01M080DA21</v>
       </c>
-      <c r="E23" s="2" t="str">
+      <c r="E23" s="64" t="str">
         <f>VLOOKUP(D23,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Lông Đền Phẳng Thép Mạ Kẽm M8 (19x1.0)</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D23,Nhập!$F$4:$F$1213)</f>
         <v>2010</v>
       </c>
-      <c r="G23" s="2">
+      <c r="G23" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D23,Xuất!$F$6:$F$1043)</f>
         <v>2000</v>
       </c>
-      <c r="H23" s="7">
+      <c r="H23" s="64">
         <f>F23-G23</f>
         <v>10</v>
       </c>
@@ -7173,23 +7192,23 @@
       <c r="C24" s="2">
         <v>19</v>
       </c>
-      <c r="D24" s="22" t="str">
+      <c r="D24" s="65" t="str">
         <f>'danh mục Vật tư'!B21</f>
         <v>BOS-06013940K0</v>
       </c>
-      <c r="E24" s="2" t="str">
+      <c r="E24" s="64" t="str">
         <f>VLOOKUP(D24,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Máy Mài Góc 750W GWS 750-100 Bosch 06013940K0</v>
       </c>
-      <c r="F24" s="2">
+      <c r="F24" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D24,Nhập!$F$4:$F$1213)</f>
         <v>2</v>
       </c>
-      <c r="G24" s="2">
+      <c r="G24" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D24,Xuất!$F$6:$F$1043)</f>
         <v>2</v>
       </c>
-      <c r="H24" s="7">
+      <c r="H24" s="64">
         <f t="shared" ref="H24:H39" si="2">F24-G24</f>
         <v>0</v>
       </c>
@@ -7204,23 +7223,23 @@
       <c r="C25" s="2">
         <v>20</v>
       </c>
-      <c r="D25" s="22" t="str">
+      <c r="D25" s="65" t="str">
         <f>'danh mục Vật tư'!B22</f>
         <v>N01M0801D21</v>
       </c>
-      <c r="E25" s="2" t="str">
+      <c r="E25" s="64" t="str">
         <f>VLOOKUP(D25,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Thép Mạ Kẽm 8.8 DIN934 M8</v>
       </c>
-      <c r="F25" s="2">
+      <c r="F25" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D25,Nhập!$F$4:$F$1213)</f>
         <v>1510</v>
       </c>
-      <c r="G25" s="2">
+      <c r="G25" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D25,Xuất!$F$6:$F$1043)</f>
         <v>1500</v>
       </c>
-      <c r="H25" s="7">
+      <c r="H25" s="64">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
@@ -7235,23 +7254,23 @@
       <c r="C26" s="2">
         <v>21</v>
       </c>
-      <c r="D26" s="22" t="str">
+      <c r="D26" s="65" t="str">
         <f>'danh mục Vật tư'!B23</f>
         <v>W01M080DA20</v>
       </c>
-      <c r="E26" s="2" t="str">
+      <c r="E26" s="64" t="str">
         <f>VLOOKUP(D26,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Lông Đền Phẳng Thép Mạ Kẽm Trắng Cr3+ M8 (19x1.0)</v>
       </c>
-      <c r="F26" s="2">
+      <c r="F26" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D26,Nhập!$F$4:$F$1213)</f>
         <v>229</v>
       </c>
-      <c r="G26" s="2">
+      <c r="G26" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D26,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H26" s="7">
+      <c r="H26" s="64">
         <f t="shared" si="2"/>
         <v>229</v>
       </c>
@@ -7266,23 +7285,23 @@
       <c r="C27" s="2">
         <v>22</v>
       </c>
-      <c r="D27" s="22" t="str">
+      <c r="D27" s="65" t="str">
         <f>'danh mục Vật tư'!B24</f>
         <v>N06M0501H00</v>
       </c>
-      <c r="E27" s="2" t="str">
+      <c r="E27" s="64" t="str">
         <f>VLOOKUP(D27,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Rút (Nutsert) Inox 304 M5</v>
       </c>
-      <c r="F27" s="2">
+      <c r="F27" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D27,Nhập!$F$4:$F$1213)</f>
         <v>1000</v>
       </c>
-      <c r="G27" s="2">
+      <c r="G27" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D27,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H27" s="7">
+      <c r="H27" s="64">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
@@ -7297,23 +7316,23 @@
       <c r="C28" s="2">
         <v>23</v>
       </c>
-      <c r="D28" s="22" t="str">
+      <c r="D28" s="65" t="str">
         <f>'danh mục Vật tư'!B25</f>
         <v>V1132010H1000</v>
       </c>
-      <c r="E28" s="2" t="str">
+      <c r="E28" s="64" t="str">
         <f>VLOOKUP(D28,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Rivet Inox 304 OD3.2x10mm (1000 Cái)</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F28" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D28,Nhập!$F$4:$F$1213)</f>
         <v>15</v>
       </c>
-      <c r="G28" s="2">
+      <c r="G28" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D28,Xuất!$F$6:$F$1043)</f>
         <v>6</v>
       </c>
-      <c r="H28" s="7">
+      <c r="H28" s="64">
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
@@ -7328,23 +7347,23 @@
       <c r="C29" s="2">
         <v>24</v>
       </c>
-      <c r="D29" s="22" t="str">
+      <c r="D29" s="65" t="str">
         <f>'danh mục Vật tư'!B26</f>
         <v>V1140010H1000</v>
       </c>
-      <c r="E29" s="2" t="str">
+      <c r="E29" s="64" t="str">
         <f>VLOOKUP(D29,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Rivet Inox 304 OD4.0x10mm (1000 Cái)</v>
       </c>
-      <c r="F29" s="2">
+      <c r="F29" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D29,Nhập!$F$4:$F$1213)</f>
         <v>8</v>
       </c>
-      <c r="G29" s="2">
+      <c r="G29" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D29,Xuất!$F$6:$F$1043)</f>
         <v>3</v>
       </c>
-      <c r="H29" s="7">
+      <c r="H29" s="64">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
@@ -7720,23 +7739,23 @@
       <c r="C42" s="2">
         <v>37</v>
       </c>
-      <c r="D42" s="22" t="str">
+      <c r="D42" s="65" t="str">
         <f>'danh mục Vật tư'!B39</f>
         <v>B01M1201025TD21</v>
       </c>
-      <c r="E42" s="2" t="str">
+      <c r="E42" s="64" t="str">
         <f>VLOOKUP(D42,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bulong Mạ Kẽm 8.8 DIN933 M12x25</v>
       </c>
-      <c r="F42" s="2">
+      <c r="F42" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D42,Nhập!$F$4:$F$1213)</f>
         <v>500</v>
       </c>
-      <c r="G42" s="2">
+      <c r="G42" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D42,Xuất!$F$6:$F$1043)</f>
         <v>100</v>
       </c>
-      <c r="H42" s="7">
+      <c r="H42" s="64">
         <f t="shared" ref="H42:H55" si="3">F42-G42</f>
         <v>400</v>
       </c>
@@ -7751,23 +7770,23 @@
       <c r="C43" s="2">
         <v>38</v>
       </c>
-      <c r="D43" s="22" t="str">
+      <c r="D43" s="65" t="str">
         <f>'danh mục Vật tư'!B40</f>
         <v>N01M1201D20</v>
       </c>
-      <c r="E43" s="2" t="str">
+      <c r="E43" s="64" t="str">
         <f>VLOOKUP(D43,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Thép Mạ Kẽm Trắng Cr3+ 8.8 DIN934 M12</v>
       </c>
-      <c r="F43" s="2">
+      <c r="F43" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D43,Nhập!$F$4:$F$1213)</f>
         <v>200</v>
       </c>
-      <c r="G43" s="2">
+      <c r="G43" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D43,Xuất!$F$6:$F$1043)</f>
         <v>100</v>
       </c>
-      <c r="H43" s="7">
+      <c r="H43" s="64">
         <f t="shared" si="3"/>
         <v>100</v>
       </c>
@@ -7782,23 +7801,23 @@
       <c r="C44" s="2">
         <v>39</v>
       </c>
-      <c r="D44" s="22" t="str">
+      <c r="D44" s="65" t="str">
         <f>'danh mục Vật tư'!B41</f>
         <v>W01M120FA2</v>
       </c>
-      <c r="E44" s="2" t="str">
+      <c r="E44" s="64" t="str">
         <f>VLOOKUP(D44,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Lông Đền Phẳng Thép Mạ Kẽm M12 (24x1.0)</v>
       </c>
-      <c r="F44" s="2">
+      <c r="F44" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D44,Nhập!$F$4:$F$1213)</f>
         <v>500</v>
       </c>
-      <c r="G44" s="2">
+      <c r="G44" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D44,Xuất!$F$6:$F$1043)</f>
         <v>200</v>
       </c>
-      <c r="H44" s="7">
+      <c r="H44" s="64">
         <f t="shared" si="3"/>
         <v>300</v>
       </c>
@@ -7813,23 +7832,23 @@
       <c r="C45" s="2">
         <v>40</v>
       </c>
-      <c r="D45" s="22" t="str">
+      <c r="D45" s="65" t="str">
         <f>'danh mục Vật tư'!B42</f>
         <v>N01M1201D21</v>
       </c>
-      <c r="E45" s="2" t="str">
+      <c r="E45" s="64" t="str">
         <f>VLOOKUP(D45,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Thép Mạ Kẽm 8.8 DIN934 M12</v>
       </c>
-      <c r="F45" s="2">
+      <c r="F45" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D45,Nhập!$F$4:$F$1213)</f>
         <v>1000</v>
       </c>
-      <c r="G45" s="2">
+      <c r="G45" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D45,Xuất!$F$6:$F$1043)</f>
         <v>200</v>
       </c>
-      <c r="H45" s="7">
+      <c r="H45" s="64">
         <f t="shared" si="3"/>
         <v>800</v>
       </c>
@@ -7844,23 +7863,23 @@
       <c r="C46" s="2">
         <v>41</v>
       </c>
-      <c r="D46" s="22" t="str">
+      <c r="D46" s="65" t="str">
         <f>'danh mục Vật tư'!B43</f>
         <v>BOS-06019H2281</v>
       </c>
-      <c r="E46" s="2" t="str">
+      <c r="E46" s="64" t="str">
         <f>VLOOKUP(D46,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Máy Vặn Vít Pin Bosch GO 3 (Kit) Bosch 06019H2281</v>
       </c>
-      <c r="F46" s="2">
+      <c r="F46" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D46,Nhập!$F$4:$F$1213)</f>
         <v>1</v>
       </c>
-      <c r="G46" s="2">
+      <c r="G46" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D46,Xuất!$F$6:$F$1043)</f>
         <v>1</v>
       </c>
-      <c r="H46" s="7">
+      <c r="H46" s="64">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -7874,23 +7893,23 @@
       <c r="C47" s="2">
         <v>42</v>
       </c>
-      <c r="D47" s="22" t="str">
+      <c r="D47" s="65" t="str">
         <f>'danh mục Vật tư'!B44</f>
         <v>N03M1001H00</v>
       </c>
-      <c r="E47" s="2" t="str">
+      <c r="E47" s="64" t="str">
         <f>VLOOKUP(D47,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Keo Inox 304 DIN985 M10</v>
       </c>
-      <c r="F47" s="2">
+      <c r="F47" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D47,Nhập!$F$4:$F$1213)</f>
         <v>1000</v>
       </c>
-      <c r="G47" s="2">
+      <c r="G47" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D47,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H47" s="7">
+      <c r="H47" s="64">
         <f t="shared" si="3"/>
         <v>1000</v>
       </c>
@@ -7904,23 +7923,23 @@
       <c r="C48" s="2">
         <v>43</v>
       </c>
-      <c r="D48" s="22" t="str">
+      <c r="D48" s="65" t="str">
         <f>'danh mục Vật tư'!B45</f>
         <v>B01M0601015TH00</v>
       </c>
-      <c r="E48" s="2" t="str">
+      <c r="E48" s="64" t="str">
         <f>VLOOKUP(D48,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bulong Inox 304 DIN933 M6x15</v>
       </c>
-      <c r="F48" s="2">
+      <c r="F48" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D48,Nhập!$F$4:$F$1213)</f>
         <v>7800</v>
       </c>
-      <c r="G48" s="2">
+      <c r="G48" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D48,Xuất!$F$6:$F$1043)</f>
         <v>7800</v>
       </c>
-      <c r="H48" s="7">
+      <c r="H48" s="64">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -7964,23 +7983,23 @@
       <c r="C50" s="2">
         <v>45</v>
       </c>
-      <c r="D50" s="22" t="str">
+      <c r="D50" s="65" t="str">
         <f>'danh mục Vật tư'!B47</f>
         <v>N01M0601H00</v>
       </c>
-      <c r="E50" s="2" t="str">
+      <c r="E50" s="64" t="str">
         <f>VLOOKUP(D50,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Inox 304 DIN934 M6</v>
       </c>
-      <c r="F50" s="2">
+      <c r="F50" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D50,Nhập!$F$4:$F$1213)</f>
         <v>15000</v>
       </c>
-      <c r="G50" s="2">
+      <c r="G50" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D50,Xuất!$F$6:$F$1043)</f>
         <v>8000</v>
       </c>
-      <c r="H50" s="7">
+      <c r="H50" s="64">
         <f t="shared" si="3"/>
         <v>7000</v>
       </c>
@@ -7994,23 +8013,23 @@
       <c r="C51" s="2">
         <v>46</v>
       </c>
-      <c r="D51" s="22" t="str">
+      <c r="D51" s="65" t="str">
         <f>'danh mục Vật tư'!B48</f>
         <v>BOS-06013960K0</v>
       </c>
-      <c r="E51" s="2" t="str">
+      <c r="E51" s="64" t="str">
         <f>VLOOKUP(D51,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Máy Mài Góc 900W GWS 900-100 Bosch 06013960K0</v>
       </c>
-      <c r="F51" s="2">
+      <c r="F51" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D51,Nhập!$F$4:$F$1213)</f>
         <v>2</v>
       </c>
-      <c r="G51" s="2">
+      <c r="G51" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D51,Xuất!$F$6:$F$1043)</f>
         <v>2</v>
       </c>
-      <c r="H51" s="7">
+      <c r="H51" s="64">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -8024,23 +8043,23 @@
       <c r="C52" s="2">
         <v>47</v>
       </c>
-      <c r="D52" s="22" t="str">
+      <c r="D52" s="65" t="str">
         <f>'danh mục Vật tư'!B49</f>
         <v>B01M1201060TD21</v>
       </c>
-      <c r="E52" s="2" t="str">
+      <c r="E52" s="64" t="str">
         <f>VLOOKUP(D52,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bulong Mạ Kẽm 8.8 DIN933 M12x60</v>
       </c>
-      <c r="F52" s="2">
+      <c r="F52" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D52,Nhập!$F$4:$F$1213)</f>
         <v>200</v>
       </c>
-      <c r="G52" s="2">
+      <c r="G52" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D52,Xuất!$F$6:$F$1043)</f>
         <v>200</v>
       </c>
-      <c r="H52" s="7">
+      <c r="H52" s="64">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -8056,23 +8075,23 @@
       <c r="C53" s="2">
         <v>48</v>
       </c>
-      <c r="D53" s="22" t="str">
+      <c r="D53" s="65" t="str">
         <f>'danh mục Vật tư'!B50</f>
         <v>W01M060BH0</v>
       </c>
-      <c r="E53" s="2" t="str">
+      <c r="E53" s="64" t="str">
         <f>VLOOKUP(D53,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Lông Đền Phẳng Inox 304 M6 (16x2.0)</v>
       </c>
-      <c r="F53" s="2">
+      <c r="F53" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D53,Nhập!$F$4:$F$1213)</f>
         <v>6000</v>
       </c>
-      <c r="G53" s="2">
+      <c r="G53" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D53,Xuất!$F$6:$F$1043)</f>
         <v>6000</v>
       </c>
-      <c r="H53" s="7">
+      <c r="H53" s="64">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -8086,23 +8105,23 @@
       <c r="C54" s="2">
         <v>49</v>
       </c>
-      <c r="D54" s="22" t="str">
+      <c r="D54" s="65" t="str">
         <f>'danh mục Vật tư'!B51</f>
         <v>W01M120AH0</v>
       </c>
-      <c r="E54" s="2" t="str">
+      <c r="E54" s="64" t="str">
         <f>VLOOKUP(D54,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Lông Đền Phẳng Inox 304 DIN125 M12</v>
       </c>
-      <c r="F54" s="2">
+      <c r="F54" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D54,Nhập!$F$4:$F$1213)</f>
         <v>3500</v>
       </c>
-      <c r="G54" s="2">
+      <c r="G54" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D54,Xuất!$F$6:$F$1043)</f>
         <v>500</v>
       </c>
-      <c r="H54" s="7">
+      <c r="H54" s="64">
         <f t="shared" si="3"/>
         <v>3000</v>
       </c>
@@ -8116,23 +8135,23 @@
       <c r="C55" s="2">
         <v>50</v>
       </c>
-      <c r="D55" s="22" t="str">
+      <c r="D55" s="65" t="str">
         <f>'danh mục Vật tư'!B52</f>
         <v>KHM08202LDI</v>
       </c>
-      <c r="E55" s="2" t="str">
+      <c r="E55" s="64" t="str">
         <f>VLOOKUP(D55,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Lông Đền Phẳng Inox 304 M8 (20x2.0)</v>
       </c>
-      <c r="F55" s="2">
+      <c r="F55" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D55,Nhập!$F$4:$F$1213)</f>
         <v>2000</v>
       </c>
-      <c r="G55" s="2">
+      <c r="G55" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D55,Xuất!$F$6:$F$1043)</f>
         <v>2000</v>
       </c>
-      <c r="H55" s="7">
+      <c r="H55" s="64">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -8146,23 +8165,23 @@
       <c r="C56" s="2">
         <v>51</v>
       </c>
-      <c r="D56" s="22" t="str">
+      <c r="D56" s="65" t="str">
         <f>'danh mục Vật tư'!B53</f>
         <v>KHBM1020BTKT</v>
       </c>
-      <c r="E56" s="2" t="str">
+      <c r="E56" s="64" t="str">
         <f>VLOOKUP(D56,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bulong chống xoay M10x20 và tán chống xoay M10 – Vật liệu thép mạ kẽm</v>
       </c>
-      <c r="F56" s="2">
+      <c r="F56" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D56,Nhập!$F$4:$F$1213)</f>
         <v>0</v>
       </c>
-      <c r="G56" s="2">
+      <c r="G56" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D56,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H56" s="7">
+      <c r="H56" s="64">
         <f t="shared" ref="H56:H66" si="4">F56-G56</f>
         <v>0</v>
       </c>
@@ -8177,23 +8196,23 @@
       <c r="C57" s="2">
         <v>52</v>
       </c>
-      <c r="D57" s="22" t="str">
+      <c r="D57" s="65" t="str">
         <f>'danh mục Vật tư'!B54</f>
         <v>B01M1001025TH00</v>
       </c>
-      <c r="E57" s="2" t="str">
+      <c r="E57" s="64" t="str">
         <f>VLOOKUP(D57,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bulong Inox 304 DIN933 M10x25</v>
       </c>
-      <c r="F57" s="2">
+      <c r="F57" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D57,Nhập!$F$4:$F$1213)</f>
         <v>900</v>
       </c>
-      <c r="G57" s="2">
+      <c r="G57" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D57,Xuất!$F$6:$F$1043)</f>
         <v>500</v>
       </c>
-      <c r="H57" s="7">
+      <c r="H57" s="64">
         <f t="shared" si="4"/>
         <v>400</v>
       </c>
@@ -8208,23 +8227,23 @@
       <c r="C58" s="2">
         <v>53</v>
       </c>
-      <c r="D58" s="22" t="str">
+      <c r="D58" s="65" t="str">
         <f>'danh mục Vật tư'!B55</f>
         <v>B01M1001040TH00</v>
       </c>
-      <c r="E58" s="2" t="str">
+      <c r="E58" s="64" t="str">
         <f>VLOOKUP(D58,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bulong Inox 304 DIN933 M10x40</v>
       </c>
-      <c r="F58" s="2">
+      <c r="F58" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D58,Nhập!$F$4:$F$1213)</f>
         <v>600</v>
       </c>
-      <c r="G58" s="2">
+      <c r="G58" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D58,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H58" s="7">
+      <c r="H58" s="64">
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
@@ -8238,23 +8257,23 @@
       <c r="C59" s="2">
         <v>54</v>
       </c>
-      <c r="D59" s="22" t="str">
+      <c r="D59" s="65" t="str">
         <f>'danh mục Vật tư'!B56</f>
         <v>N01M1001H00</v>
       </c>
-      <c r="E59" s="2" t="str">
+      <c r="E59" s="64" t="str">
         <f>VLOOKUP(D59,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Inox 304 DIN934 M10</v>
       </c>
-      <c r="F59" s="2">
+      <c r="F59" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D59,Nhập!$F$4:$F$1213)</f>
         <v>2400</v>
       </c>
-      <c r="G59" s="2">
+      <c r="G59" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D59,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H59" s="7">
+      <c r="H59" s="64">
         <f t="shared" si="4"/>
         <v>2400</v>
       </c>
@@ -8268,23 +8287,23 @@
       <c r="C60" s="2">
         <v>55</v>
       </c>
-      <c r="D60" s="22" t="str">
+      <c r="D60" s="65" t="str">
         <f>'danh mục Vật tư'!B57</f>
         <v>W01M100AH0</v>
       </c>
-      <c r="E60" s="2" t="str">
+      <c r="E60" s="64" t="str">
         <f>VLOOKUP(D60,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Lông Đền Phẳng Inox 304 DIN125 M10</v>
       </c>
-      <c r="F60" s="2">
+      <c r="F60" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D60,Nhập!$F$4:$F$1213)</f>
         <v>10000</v>
       </c>
-      <c r="G60" s="2">
+      <c r="G60" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D60,Xuất!$F$6:$F$1043)</f>
         <v>5000</v>
       </c>
-      <c r="H60" s="7">
+      <c r="H60" s="64">
         <f t="shared" si="4"/>
         <v>5000</v>
       </c>
@@ -8298,22 +8317,22 @@
       <c r="C61" s="2">
         <v>56</v>
       </c>
-      <c r="D61" s="22" t="s">
+      <c r="D61" s="65" t="s">
         <v>189</v>
       </c>
-      <c r="E61" s="2" t="str">
+      <c r="E61" s="64" t="str">
         <f>VLOOKUP(D61,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Lông Đền Phẳng Inox 304 DIN9021A M8</v>
       </c>
-      <c r="F61" s="2">
+      <c r="F61" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D61,Nhập!$F$4:$F$1213)</f>
         <v>3500</v>
       </c>
-      <c r="G61" s="2">
+      <c r="G61" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D61,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H61" s="7">
+      <c r="H61" s="64">
         <f t="shared" si="4"/>
         <v>3500</v>
       </c>
@@ -8539,28 +8558,28 @@
       <c r="C69" s="2">
         <v>64</v>
       </c>
-      <c r="D69" s="22" t="str">
+      <c r="D69" s="65" t="str">
         <f>'danh mục Vật tư'!B66</f>
         <v>SAT-09105A</v>
       </c>
-      <c r="E69" s="2" t="str">
+      <c r="E69" s="64" t="str">
         <f>VLOOKUP(D69,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v xml:space="preserve">
 Bộ Cây Vặn Lục Giác Bi Loại Dài 9 Chi Tiết - Hệ Mét SATA 09105A</v>
       </c>
-      <c r="F69" s="2">
+      <c r="F69" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D69,Nhập!$F$4:$F$1213)</f>
         <v>1</v>
       </c>
-      <c r="G69" s="2">
+      <c r="G69" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D69,Xuất!$F$6:$F$1043)</f>
         <v>1</v>
       </c>
-      <c r="H69" s="7">
+      <c r="H69" s="64">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I69" s="22" t="str">
+      <c r="I69" s="65" t="str">
         <f>VLOOKUP(D69,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Bộ</v>
       </c>
@@ -8570,27 +8589,27 @@
       <c r="C70" s="2">
         <v>65</v>
       </c>
-      <c r="D70" s="22" t="str">
+      <c r="D70" s="65" t="str">
         <f>'danh mục Vật tư'!B67</f>
         <v>HD100A060</v>
       </c>
-      <c r="E70" s="2" t="str">
+      <c r="E70" s="64" t="str">
         <f>VLOOKUP(D70,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Đá Nhám Xếp Hải Dương CN A60-D100</v>
       </c>
-      <c r="F70" s="2">
+      <c r="F70" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D70,Nhập!$F$4:$F$1213)</f>
         <v>30</v>
       </c>
-      <c r="G70" s="2">
+      <c r="G70" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D70,Xuất!$F$6:$F$1043)</f>
         <v>30</v>
       </c>
-      <c r="H70" s="7">
+      <c r="H70" s="64">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I70" s="22" t="str">
+      <c r="I70" s="65" t="str">
         <f>VLOOKUP(D70,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Cái</v>
       </c>
@@ -8600,27 +8619,27 @@
       <c r="C71" s="2">
         <v>66</v>
       </c>
-      <c r="D71" s="22" t="str">
+      <c r="D71" s="65" t="str">
         <f>'danh mục Vật tư'!B68</f>
         <v>KOY-6201-ZZ</v>
       </c>
-      <c r="E71" s="2" t="str">
+      <c r="E71" s="64" t="str">
         <f>VLOOKUP(D71,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Vòng Bi Cầu Rãnh Sâu KOYO 6201 ZZ (12x32x10) Hai Nắp Thép</v>
       </c>
-      <c r="F71" s="2">
+      <c r="F71" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D71,Nhập!$F$4:$F$1213)</f>
         <v>2</v>
       </c>
-      <c r="G71" s="2">
+      <c r="G71" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D71,Xuất!$F$6:$F$1043)</f>
         <v>2</v>
       </c>
-      <c r="H71" s="7">
+      <c r="H71" s="64">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I71" s="22" t="str">
+      <c r="I71" s="65" t="str">
         <f>VLOOKUP(D71,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Cái</v>
       </c>
@@ -8630,27 +8649,27 @@
       <c r="C72" s="2">
         <v>67</v>
       </c>
-      <c r="D72" s="22" t="str">
+      <c r="D72" s="65" t="str">
         <f>'danh mục Vật tư'!B69</f>
         <v>KOY-6202-ZZ</v>
       </c>
-      <c r="E72" s="2" t="str">
+      <c r="E72" s="64" t="str">
         <f>VLOOKUP(D72,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Vòng Bi Cầu Rãnh Sâu KOYO 6202 ZZ (15x35x11) Hai Nắp Thép</v>
       </c>
-      <c r="F72" s="2">
+      <c r="F72" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D72,Nhập!$F$4:$F$1213)</f>
         <v>2</v>
       </c>
-      <c r="G72" s="2">
+      <c r="G72" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D72,Xuất!$F$6:$F$1043)</f>
         <v>2</v>
       </c>
-      <c r="H72" s="7">
+      <c r="H72" s="64">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I72" s="22" t="str">
+      <c r="I72" s="65" t="str">
         <f>VLOOKUP(D72,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Cái</v>
       </c>
@@ -8660,28 +8679,28 @@
       <c r="C73" s="2">
         <v>68</v>
       </c>
-      <c r="D73" s="22" t="str">
+      <c r="D73" s="65" t="str">
         <f>'danh mục Vật tư'!B70</f>
         <v>SAT-09106</v>
       </c>
-      <c r="E73" s="2" t="str">
+      <c r="E73" s="64" t="str">
         <f>VLOOKUP(D73,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v xml:space="preserve">
 Bộ Cây Vặn Lục Giác Bi Loại Dài 12 Chi Tiết - Hệ inch SATA 09106</v>
       </c>
-      <c r="F73" s="2">
+      <c r="F73" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D73,Nhập!$F$4:$F$1213)</f>
         <v>1</v>
       </c>
-      <c r="G73" s="2">
+      <c r="G73" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D73,Xuất!$F$6:$F$1043)</f>
         <v>1</v>
       </c>
-      <c r="H73" s="7">
+      <c r="H73" s="64">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I73" s="22" t="str">
+      <c r="I73" s="65" t="str">
         <f>VLOOKUP(D73,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Bộ</v>
       </c>
@@ -8691,27 +8710,27 @@
       <c r="C74" s="2">
         <v>69</v>
       </c>
-      <c r="D74" s="22" t="str">
+      <c r="D74" s="65" t="str">
         <f>'danh mục Vật tư'!B71</f>
         <v>SAT-09702</v>
       </c>
-      <c r="E74" s="2" t="str">
+      <c r="E74" s="64" t="str">
         <f>VLOOKUP(D74,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bộ Cây Vặn Lục Giác Sao Loại Dài, 9 Chi Tiết SATA 09702</v>
       </c>
-      <c r="F74" s="2">
+      <c r="F74" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D74,Nhập!$F$4:$F$1213)</f>
         <v>1</v>
       </c>
-      <c r="G74" s="2">
+      <c r="G74" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D74,Xuất!$F$6:$F$1043)</f>
         <v>1</v>
       </c>
-      <c r="H74" s="7">
+      <c r="H74" s="64">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I74" s="22" t="str">
+      <c r="I74" s="65" t="str">
         <f>VLOOKUP(D74,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Bộ</v>
       </c>
@@ -8721,27 +8740,27 @@
       <c r="C75" s="2">
         <v>70</v>
       </c>
-      <c r="D75" s="22" t="str">
+      <c r="D75" s="65" t="str">
         <f>'danh mục Vật tư'!B72</f>
         <v>N06M0601H00</v>
       </c>
-      <c r="E75" s="2" t="str">
+      <c r="E75" s="64" t="str">
         <f>VLOOKUP(D75,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Tán Rút (Nutsert) Inox 304 M6</v>
       </c>
-      <c r="F75" s="2">
+      <c r="F75" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D75,Nhập!$F$4:$F$1213)</f>
         <v>1000</v>
       </c>
-      <c r="G75" s="2">
+      <c r="G75" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D75,Xuất!$F$6:$F$1043)</f>
         <v>200</v>
       </c>
-      <c r="H75" s="7">
+      <c r="H75" s="64">
         <f t="shared" si="5"/>
         <v>800</v>
       </c>
-      <c r="I75" s="22" t="str">
+      <c r="I75" s="65" t="str">
         <f>VLOOKUP(D75,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Cái</v>
       </c>
@@ -8751,27 +8770,27 @@
       <c r="C76" s="2">
         <v>71</v>
       </c>
-      <c r="D76" s="22" t="str">
+      <c r="D76" s="65" t="str">
         <f>'danh mục Vật tư'!B73</f>
         <v>WW-VPBGM860</v>
       </c>
-      <c r="E76" s="2" t="str">
+      <c r="E76" s="64" t="str">
         <f>VLOOKUP(D76,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Vít Phong Bắn Gỗ M8x60</v>
       </c>
-      <c r="F76" s="2">
+      <c r="F76" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D76,Nhập!$F$4:$F$1213)</f>
         <v>500</v>
       </c>
-      <c r="G76" s="2">
+      <c r="G76" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D76,Xuất!$F$6:$F$1043)</f>
         <v>500</v>
       </c>
-      <c r="H76" s="7">
+      <c r="H76" s="64">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I76" s="22" t="str">
+      <c r="I76" s="65" t="str">
         <f>VLOOKUP(D76,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Cái</v>
       </c>
@@ -8781,27 +8800,27 @@
       <c r="C77" s="2">
         <v>72</v>
       </c>
-      <c r="D77" s="22" t="str">
+      <c r="D77" s="65" t="str">
         <f>'danh mục Vật tư'!B74</f>
         <v>WW-BLXM1260</v>
       </c>
-      <c r="E77" s="2" t="str">
+      <c r="E77" s="64" t="str">
         <f>VLOOKUP(D77,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bu lông xi 12x60</v>
       </c>
-      <c r="F77" s="2">
+      <c r="F77" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D77,Nhập!$F$4:$F$1213)</f>
         <v>500</v>
       </c>
-      <c r="G77" s="2">
+      <c r="G77" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D77,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H77" s="7">
+      <c r="H77" s="64">
         <f t="shared" si="5"/>
         <v>500</v>
       </c>
-      <c r="I77" s="22" t="str">
+      <c r="I77" s="65" t="str">
         <f>VLOOKUP(D77,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Cái</v>
       </c>
@@ -8811,27 +8830,27 @@
       <c r="C78" s="2">
         <v>73</v>
       </c>
-      <c r="D78" s="22" t="str">
+      <c r="D78" s="65" t="str">
         <f>'danh mục Vật tư'!B75</f>
         <v>WW- MKIT20</v>
       </c>
-      <c r="E78" s="2" t="str">
+      <c r="E78" s="64" t="str">
         <f>VLOOKUP(D78,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Mũi khoét inox top 1 20mm (10c/HG)</v>
       </c>
-      <c r="F78" s="2">
+      <c r="F78" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D78,Nhập!$F$4:$F$1213)</f>
         <v>10</v>
       </c>
-      <c r="G78" s="2">
+      <c r="G78" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D78,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H78" s="7">
+      <c r="H78" s="64">
         <f t="shared" si="5"/>
         <v>10</v>
       </c>
-      <c r="I78" s="22" t="str">
+      <c r="I78" s="65" t="str">
         <f>VLOOKUP(D78,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>Cái</v>
       </c>
@@ -8841,27 +8860,27 @@
       <c r="C79" s="2">
         <v>74</v>
       </c>
-      <c r="D79" s="22" t="str">
+      <c r="D79" s="65" t="str">
         <f>'danh mục Vật tư'!B76</f>
         <v>WW-RVNM412</v>
       </c>
-      <c r="E79" s="2" t="str">
+      <c r="E79" s="64" t="str">
         <f>VLOOKUP(D79,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Ri vê 4x12 (bịch 1kg - 600c/BC - Nhôm)</v>
       </c>
-      <c r="F79" s="2">
+      <c r="F79" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D79,Nhập!$F$4:$F$1213)</f>
         <v>10</v>
       </c>
-      <c r="G79" s="2">
+      <c r="G79" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D79,Xuất!$F$6:$F$1043)</f>
         <v>0</v>
       </c>
-      <c r="H79" s="7">
+      <c r="H79" s="64">
         <f t="shared" si="5"/>
         <v>10</v>
       </c>
-      <c r="I79" s="22" t="str">
+      <c r="I79" s="65" t="str">
         <f>VLOOKUP(D79,'danh mục Vật tư'!$B$3:$H$173,7,0)</f>
         <v>bịch</v>
       </c>
@@ -8871,23 +8890,23 @@
       <c r="C80" s="2">
         <v>75</v>
       </c>
-      <c r="D80" s="22" t="str">
+      <c r="D80" s="65" t="str">
         <f>'danh mục Vật tư'!B77</f>
         <v>KH-BLIM615</v>
       </c>
-      <c r="E80" s="2" t="str">
+      <c r="E80" s="64" t="str">
         <f>VLOOKUP(D80,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Bu lông inox 304 size 6x15mm</v>
       </c>
-      <c r="F80" s="2">
+      <c r="F80" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D80,Nhập!$F$4:$F$1213)</f>
         <v>200</v>
       </c>
-      <c r="G80" s="2">
+      <c r="G80" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D80,Xuất!$F$6:$F$1043)</f>
         <v>200</v>
       </c>
-      <c r="H80" s="7">
+      <c r="H80" s="64">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -8901,23 +8920,23 @@
       <c r="C81" s="2">
         <v>76</v>
       </c>
-      <c r="D81" s="22" t="str">
+      <c r="D81" s="65" t="str">
         <f>'danh mục Vật tư'!B78</f>
         <v>KH-VDPIM6162</v>
       </c>
-      <c r="E81" s="2" t="str">
+      <c r="E81" s="64" t="str">
         <f>VLOOKUP(D81,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Vòng đệm phẳng inox 304 size 6x16x2mm</v>
       </c>
-      <c r="F81" s="2">
+      <c r="F81" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D81,Nhập!$F$4:$F$1213)</f>
         <v>10000</v>
       </c>
-      <c r="G81" s="2">
+      <c r="G81" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D81,Xuất!$F$6:$F$1043)</f>
         <v>10000</v>
       </c>
-      <c r="H81" s="7">
+      <c r="H81" s="64">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -8931,23 +8950,23 @@
       <c r="C82" s="2">
         <v>77</v>
       </c>
-      <c r="D82" s="22" t="str">
+      <c r="D82" s="65" t="str">
         <f>'danh mục Vật tư'!B79</f>
         <v>KH-VDPIM8202</v>
       </c>
-      <c r="E82" s="2" t="str">
+      <c r="E82" s="64" t="str">
         <f>VLOOKUP(D82,'danh mục Vật tư'!$B$3:$G$173,2,0)</f>
         <v>Vòng đệm phẳng inox 304 size 8x20x2mm</v>
       </c>
-      <c r="F82" s="2">
+      <c r="F82" s="64">
         <f>SUMIF(Nhập!$D$4:$D$1131,Tồn!D82,Nhập!$F$4:$F$1213)</f>
         <v>1000</v>
       </c>
-      <c r="G82" s="2">
+      <c r="G82" s="64">
         <f>SUMIF(Xuất!$D$6:$D$265,Tồn!D82,Xuất!$F$6:$F$1043)</f>
         <v>1000</v>
       </c>
-      <c r="H82" s="7">
+      <c r="H82" s="64">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -10367,12 +10386,12 @@
   <sheetData>
     <row r="1" spans="1:9" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="15"/>
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="61" t="s">
         <v>128</v>
       </c>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
       <c r="F1" s="20"/>
       <c r="G1" s="42"/>
       <c r="H1" s="21"/>
@@ -23165,293 +23184,293 @@
       <c r="G1" s="63"/>
     </row>
     <row r="2" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="55" t="s">
         <v>240</v>
       </c>
-      <c r="C2" s="57" t="s">
+      <c r="C2" s="55" t="s">
         <v>239</v>
       </c>
-      <c r="D2" s="58" t="s">
+      <c r="D2" s="56" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="58" t="s">
+      <c r="E2" s="56" t="s">
         <v>244</v>
       </c>
-      <c r="F2" s="58" t="s">
+      <c r="F2" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="58" t="s">
+      <c r="G2" s="56" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="59">
+      <c r="A3" s="57">
         <v>1</v>
       </c>
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="57" t="s">
         <v>242</v>
       </c>
-      <c r="C3" s="59" t="s">
+      <c r="C3" s="57" t="s">
         <v>246</v>
       </c>
-      <c r="D3" s="60" t="s">
+      <c r="D3" s="58" t="s">
         <v>245</v>
       </c>
-      <c r="E3" s="60" t="s">
+      <c r="E3" s="58" t="s">
         <v>243</v>
       </c>
-      <c r="F3" s="60" t="s">
+      <c r="F3" s="58" t="s">
         <v>247</v>
       </c>
-      <c r="G3" s="61" t="s">
+      <c r="G3" s="59" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="59"/>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="60"/>
-      <c r="G4" s="60"/>
+      <c r="A4" s="57"/>
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
     </row>
     <row r="5" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="59"/>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="62"/>
-      <c r="F5" s="60"/>
-      <c r="G5" s="60"/>
+      <c r="A5" s="57"/>
+      <c r="B5" s="57"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="58"/>
+      <c r="G5" s="58"/>
     </row>
     <row r="6" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="59"/>
-      <c r="B6" s="59"/>
-      <c r="C6" s="59"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="60"/>
-      <c r="G6" s="60"/>
+      <c r="A6" s="57"/>
+      <c r="B6" s="57"/>
+      <c r="C6" s="57"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58"/>
     </row>
     <row r="7" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="59"/>
-      <c r="B7" s="59"/>
-      <c r="C7" s="59"/>
-      <c r="D7" s="60"/>
-      <c r="E7" s="62"/>
-      <c r="F7" s="60"/>
-      <c r="G7" s="60"/>
+      <c r="A7" s="57"/>
+      <c r="B7" s="57"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="60"/>
+      <c r="F7" s="58"/>
+      <c r="G7" s="58"/>
     </row>
     <row r="8" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="59"/>
-      <c r="B8" s="59"/>
-      <c r="C8" s="59"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="60"/>
-      <c r="G8" s="60"/>
+      <c r="A8" s="57"/>
+      <c r="B8" s="57"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="60"/>
+      <c r="F8" s="58"/>
+      <c r="G8" s="58"/>
     </row>
     <row r="9" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="59"/>
-      <c r="B9" s="59"/>
-      <c r="C9" s="59"/>
-      <c r="D9" s="60"/>
-      <c r="E9" s="62"/>
-      <c r="F9" s="60"/>
-      <c r="G9" s="60"/>
+      <c r="A9" s="57"/>
+      <c r="B9" s="57"/>
+      <c r="C9" s="57"/>
+      <c r="D9" s="58"/>
+      <c r="E9" s="60"/>
+      <c r="F9" s="58"/>
+      <c r="G9" s="58"/>
     </row>
     <row r="10" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="59"/>
-      <c r="B10" s="59"/>
-      <c r="C10" s="59"/>
-      <c r="D10" s="60"/>
-      <c r="E10" s="62"/>
-      <c r="F10" s="60"/>
-      <c r="G10" s="60"/>
+      <c r="A10" s="57"/>
+      <c r="B10" s="57"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="58"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="58"/>
+      <c r="G10" s="58"/>
     </row>
     <row r="11" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="59"/>
-      <c r="B11" s="59"/>
-      <c r="C11" s="59"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="62"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
+      <c r="A11" s="57"/>
+      <c r="B11" s="57"/>
+      <c r="C11" s="57"/>
+      <c r="D11" s="58"/>
+      <c r="E11" s="60"/>
+      <c r="F11" s="58"/>
+      <c r="G11" s="58"/>
     </row>
     <row r="12" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="59"/>
-      <c r="B12" s="59"/>
-      <c r="C12" s="59"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
+      <c r="A12" s="57"/>
+      <c r="B12" s="57"/>
+      <c r="C12" s="57"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="58"/>
+      <c r="G12" s="58"/>
     </row>
     <row r="13" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="59"/>
-      <c r="B13" s="59"/>
-      <c r="C13" s="59"/>
-      <c r="D13" s="60"/>
-      <c r="E13" s="62"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="60"/>
+      <c r="A13" s="57"/>
+      <c r="B13" s="57"/>
+      <c r="C13" s="57"/>
+      <c r="D13" s="58"/>
+      <c r="E13" s="60"/>
+      <c r="F13" s="58"/>
+      <c r="G13" s="58"/>
     </row>
     <row r="14" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="59"/>
-      <c r="B14" s="59"/>
-      <c r="C14" s="59"/>
-      <c r="D14" s="60"/>
-      <c r="E14" s="62"/>
-      <c r="F14" s="60"/>
-      <c r="G14" s="60"/>
+      <c r="A14" s="57"/>
+      <c r="B14" s="57"/>
+      <c r="C14" s="57"/>
+      <c r="D14" s="58"/>
+      <c r="E14" s="60"/>
+      <c r="F14" s="58"/>
+      <c r="G14" s="58"/>
     </row>
     <row r="15" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="59"/>
-      <c r="B15" s="59"/>
-      <c r="C15" s="59"/>
-      <c r="D15" s="60"/>
-      <c r="E15" s="62"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="60"/>
+      <c r="A15" s="57"/>
+      <c r="B15" s="57"/>
+      <c r="C15" s="57"/>
+      <c r="D15" s="58"/>
+      <c r="E15" s="60"/>
+      <c r="F15" s="58"/>
+      <c r="G15" s="58"/>
     </row>
     <row r="16" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="59"/>
-      <c r="B16" s="59"/>
-      <c r="C16" s="59"/>
-      <c r="D16" s="60"/>
-      <c r="E16" s="62"/>
-      <c r="F16" s="60"/>
-      <c r="G16" s="60"/>
+      <c r="A16" s="57"/>
+      <c r="B16" s="57"/>
+      <c r="C16" s="57"/>
+      <c r="D16" s="58"/>
+      <c r="E16" s="60"/>
+      <c r="F16" s="58"/>
+      <c r="G16" s="58"/>
     </row>
     <row r="17" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="59"/>
-      <c r="B17" s="59"/>
-      <c r="C17" s="59"/>
-      <c r="D17" s="60"/>
-      <c r="E17" s="62"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="60"/>
+      <c r="A17" s="57"/>
+      <c r="B17" s="57"/>
+      <c r="C17" s="57"/>
+      <c r="D17" s="58"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="58"/>
+      <c r="G17" s="58"/>
     </row>
     <row r="18" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="59"/>
-      <c r="B18" s="59"/>
-      <c r="C18" s="59"/>
-      <c r="D18" s="60"/>
-      <c r="E18" s="62"/>
-      <c r="F18" s="60"/>
-      <c r="G18" s="60"/>
+      <c r="A18" s="57"/>
+      <c r="B18" s="57"/>
+      <c r="C18" s="57"/>
+      <c r="D18" s="58"/>
+      <c r="E18" s="60"/>
+      <c r="F18" s="58"/>
+      <c r="G18" s="58"/>
     </row>
     <row r="19" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="59"/>
-      <c r="B19" s="59"/>
-      <c r="C19" s="59"/>
-      <c r="D19" s="60"/>
-      <c r="E19" s="62"/>
-      <c r="F19" s="60"/>
-      <c r="G19" s="60"/>
+      <c r="A19" s="57"/>
+      <c r="B19" s="57"/>
+      <c r="C19" s="57"/>
+      <c r="D19" s="58"/>
+      <c r="E19" s="60"/>
+      <c r="F19" s="58"/>
+      <c r="G19" s="58"/>
     </row>
     <row r="20" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="59"/>
-      <c r="B20" s="59"/>
-      <c r="C20" s="59"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="62"/>
-      <c r="F20" s="60"/>
-      <c r="G20" s="60"/>
+      <c r="A20" s="57"/>
+      <c r="B20" s="57"/>
+      <c r="C20" s="57"/>
+      <c r="D20" s="58"/>
+      <c r="E20" s="60"/>
+      <c r="F20" s="58"/>
+      <c r="G20" s="58"/>
     </row>
     <row r="21" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="59"/>
-      <c r="B21" s="59"/>
-      <c r="C21" s="59"/>
-      <c r="D21" s="60"/>
-      <c r="E21" s="62"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="60"/>
+      <c r="A21" s="57"/>
+      <c r="B21" s="57"/>
+      <c r="C21" s="57"/>
+      <c r="D21" s="58"/>
+      <c r="E21" s="60"/>
+      <c r="F21" s="58"/>
+      <c r="G21" s="58"/>
     </row>
     <row r="22" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="59"/>
-      <c r="B22" s="59"/>
-      <c r="C22" s="59"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="62"/>
-      <c r="F22" s="60"/>
-      <c r="G22" s="60"/>
+      <c r="A22" s="57"/>
+      <c r="B22" s="57"/>
+      <c r="C22" s="57"/>
+      <c r="D22" s="58"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="58"/>
+      <c r="G22" s="58"/>
     </row>
     <row r="23" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="59"/>
-      <c r="B23" s="59"/>
-      <c r="C23" s="59"/>
-      <c r="D23" s="60"/>
-      <c r="E23" s="62"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
+      <c r="A23" s="57"/>
+      <c r="B23" s="57"/>
+      <c r="C23" s="57"/>
+      <c r="D23" s="58"/>
+      <c r="E23" s="60"/>
+      <c r="F23" s="58"/>
+      <c r="G23" s="58"/>
     </row>
     <row r="24" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="59"/>
-      <c r="B24" s="59"/>
-      <c r="C24" s="59"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="60"/>
+      <c r="A24" s="57"/>
+      <c r="B24" s="57"/>
+      <c r="C24" s="57"/>
+      <c r="D24" s="58"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="58"/>
+      <c r="G24" s="58"/>
     </row>
     <row r="25" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="59"/>
-      <c r="B25" s="59"/>
-      <c r="C25" s="59"/>
-      <c r="D25" s="60"/>
-      <c r="E25" s="62"/>
-      <c r="F25" s="60"/>
-      <c r="G25" s="60"/>
+      <c r="A25" s="57"/>
+      <c r="B25" s="57"/>
+      <c r="C25" s="57"/>
+      <c r="D25" s="58"/>
+      <c r="E25" s="60"/>
+      <c r="F25" s="58"/>
+      <c r="G25" s="58"/>
     </row>
     <row r="26" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="59"/>
-      <c r="B26" s="59"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="60"/>
-      <c r="E26" s="62"/>
-      <c r="F26" s="60"/>
-      <c r="G26" s="60"/>
+      <c r="A26" s="57"/>
+      <c r="B26" s="57"/>
+      <c r="C26" s="57"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="60"/>
+      <c r="F26" s="58"/>
+      <c r="G26" s="58"/>
     </row>
     <row r="27" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="59"/>
-      <c r="B27" s="59"/>
-      <c r="C27" s="59"/>
-      <c r="D27" s="60"/>
-      <c r="E27" s="62"/>
-      <c r="F27" s="60"/>
-      <c r="G27" s="60"/>
+      <c r="A27" s="57"/>
+      <c r="B27" s="57"/>
+      <c r="C27" s="57"/>
+      <c r="D27" s="58"/>
+      <c r="E27" s="60"/>
+      <c r="F27" s="58"/>
+      <c r="G27" s="58"/>
     </row>
     <row r="28" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="59"/>
-      <c r="B28" s="59"/>
-      <c r="C28" s="59"/>
-      <c r="D28" s="60"/>
-      <c r="E28" s="62"/>
-      <c r="F28" s="60"/>
-      <c r="G28" s="60"/>
+      <c r="A28" s="57"/>
+      <c r="B28" s="57"/>
+      <c r="C28" s="57"/>
+      <c r="D28" s="58"/>
+      <c r="E28" s="60"/>
+      <c r="F28" s="58"/>
+      <c r="G28" s="58"/>
     </row>
     <row r="29" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="59"/>
-      <c r="B29" s="59"/>
-      <c r="C29" s="59"/>
-      <c r="D29" s="60"/>
-      <c r="E29" s="62"/>
-      <c r="F29" s="60"/>
-      <c r="G29" s="60"/>
+      <c r="A29" s="57"/>
+      <c r="B29" s="57"/>
+      <c r="C29" s="57"/>
+      <c r="D29" s="58"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="58"/>
+      <c r="G29" s="58"/>
     </row>
     <row r="30" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="59"/>
-      <c r="B30" s="59"/>
-      <c r="C30" s="59"/>
-      <c r="D30" s="60"/>
-      <c r="E30" s="62"/>
-      <c r="F30" s="60"/>
-      <c r="G30" s="60"/>
+      <c r="A30" s="57"/>
+      <c r="B30" s="57"/>
+      <c r="C30" s="57"/>
+      <c r="D30" s="58"/>
+      <c r="E30" s="60"/>
+      <c r="F30" s="58"/>
+      <c r="G30" s="58"/>
     </row>
     <row r="31" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A31" s="29"/>

</xml_diff>